<commit_message>
metodologia: N/A e Blocked contam como executados; resumo do demo alinhado
Decisao do utilizador (24.09.2026): executado = todo o caso fora de Por
testar; % executada = executados / total. O resumo do demo excluia os N/A
((total - por testar - N/A) / (total - N/A)) e divergia do painel.

- metodologia 16.3: definicao de Total executado.
- demo: gerar_workbook.py com =IFERROR((B-C)/B,0) e nota; workbook
  regenerado (comparado celula a celula: so as 4 formulas e a nota mudaram).
- verificado numa copia com 1 Pass + 1 N/A: resumo 2/7 e 2/18, painel 2/18,
  resumo vs contagem direta bate certo.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/demo/workbook/plano-demo.xlsx
+++ b/examples/demo/workbook/plano-demo.xlsx
@@ -524,7 +524,7 @@
         <v/>
       </c>
       <c r="H4" s="3">
-        <f>IFERROR((B4-C4-G4)/(B4-G4),0)</f>
+        <f>IFERROR((B4-C4)/B4,0)</f>
         <v/>
       </c>
     </row>
@@ -559,7 +559,7 @@
         <v/>
       </c>
       <c r="H5" s="3">
-        <f>IFERROR((B5-C5-G5)/(B5-G5),0)</f>
+        <f>IFERROR((B5-C5)/B5,0)</f>
         <v/>
       </c>
     </row>
@@ -594,7 +594,7 @@
         <v/>
       </c>
       <c r="H6" s="3">
-        <f>IFERROR((B6-C6-G6)/(B6-G6),0)</f>
+        <f>IFERROR((B6-C6)/B6,0)</f>
         <v/>
       </c>
     </row>
@@ -629,14 +629,14 @@
         <v/>
       </c>
       <c r="H7" s="3">
-        <f>IFERROR((B7-C7-G7)/(B7-G7),0)</f>
+        <f>IFERROR((B7-C7)/B7,0)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>% Executado exclui os casos N/A.</t>
+          <t>% Executado = casos fora de Por testar (N/A e Blocked contam como executados).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
2.3: primeiro lote de UI no demo (8 casos aprovados)
- runs/lote_20260924_ui01.json: 6 Pass, CT-PROD-005 Fail -> BUG-3
  (problem_user: os 6 produtos com a mesma imagem); CT-LOGIN-006 em Duvida
  (login com o erro certo, mas o URL fica /inventory.html), fora do lote.
- Aplicado pelo adaptador: cross-check limpo, recalculo OK, resumo bate certo.
- Executado com a biblioteca Playwright no Chrome (o Playwright MCP nao estava
  disponivel na sessao); diferenca registada.
- contexto.md do demo atualizado (duvida, proximos passos, BUG-4 a seguir).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/demo/workbook/plano-demo.xlsx
+++ b/examples/demo/workbook/plano-demo.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="258">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="273">
   <si>
     <t xml:space="preserve">Demo QA — saucedemo.com (site público de prática)</t>
   </si>
@@ -137,6 +137,9 @@
     <t xml:space="preserve">Abre a página "Products" (/inventory.html).</t>
   </si>
   <si>
+    <t xml:space="preserve">Abre /inventory.html com o título "Products".</t>
+  </si>
+  <si>
     <t xml:space="preserve">CT-LOGIN-002</t>
   </si>
   <si>
@@ -150,6 +153,9 @@
   </si>
   <si>
     <t xml:space="preserve">Mostra o erro "Epic sadface: Sorry, this user has been locked out." e fica na página de login.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mostra "Epic sadface: Sorry, this user has been locked out."; fica em /.</t>
   </si>
   <si>
     <t xml:space="preserve">CT-LOGIN-003</t>
@@ -169,6 +175,9 @@
   </si>
   <si>
     <t xml:space="preserve">Mostra o erro "Epic sadface: Username is required".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mostra "Epic sadface: Username is required"; fica em /.</t>
   </si>
   <si>
     <t xml:space="preserve">CT-LOGIN-004</t>
@@ -247,6 +256,9 @@
     <t xml:space="preserve">São apresentados 6 produtos, cada um com nome, descrição, preço, imagem e botão "Add to cart".</t>
   </si>
   <si>
+    <t xml:space="preserve">6 produtos, todos com nome, descrição, preço, imagem e botão "Add to cart".</t>
+  </si>
+  <si>
     <t xml:space="preserve">CT-PROD-002</t>
   </si>
   <si>
@@ -257,6 +269,9 @@
   </si>
   <si>
     <t xml:space="preserve">Os produtos ficam por ordem crescente de preço.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preços por ordem crescente: 7.99, 9.99, 15.99, 15.99, 29.99, 49.99.</t>
   </si>
   <si>
     <t xml:space="preserve">CT-PROD-003</t>
@@ -303,6 +318,12 @@
     <t xml:space="preserve">Cada produto mostra a sua própria imagem, igual à apresentada ao standard_user.</t>
   </si>
   <si>
+    <t xml:space="preserve">Os 6 produtos mostram a mesma imagem (/assets/sl-404-….jpg); no standard_user cada produto tem a sua.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2026-09-24, lote_20260924_ui01] Defeito novo: BUG-3.</t>
+  </si>
+  <si>
     <t xml:space="preserve">CT-CHK-001</t>
   </si>
   <si>
@@ -313,6 +334,9 @@
   </si>
   <si>
     <t xml:space="preserve">O contador do carrinho mostra 1 e o botão do produto passa a "Remove".</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Contador do carrinho = 1; botão passa a "Remove" (produto removido a seguir, para limpar).</t>
   </si>
   <si>
     <t xml:space="preserve">CT-CHK-002</t>
@@ -773,10 +797,22 @@
 Evidência: runs/a11y_20260924_01.json (campo titulo de cada página).</t>
   </si>
   <si>
+    <t xml:space="preserve">BUG-3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">problem_user: todos os produtos mostram a mesma imagem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ambiente: saucedemo.com (teste), Chrome 153 via biblioteca Playwright (não o Playwright MCP, que não estava disponível nesta sessão). Role: problem_user.
+Passos: login com problem_user; observar a imagem de cada produto em Products; repetir com standard_user.
+Esperado: cada produto com a sua própria imagem, igual à apresentada ao standard_user.
+Observado: os 6 produtos mostram a mesma imagem (/assets/sl-404-….jpg); com standard_user as 6 imagens são diferentes e correspondem a cada produto.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Defeitos ativos (regenerado pelo adaptador — não editar à mão)</t>
   </si>
   <si>
-    <t xml:space="preserve">2 abertos (0 Crítica, 0 Alta, 1 Média, 1 Baixa) · 0 fechados · atualizado a 24.09.2026</t>
+    <t xml:space="preserve">3 abertos (0 Crítica, 0 Alta, 2 Média, 1 Baixa) · 0 fechados · atualizado a 24.09.2026</t>
   </si>
   <si>
     <t xml:space="preserve">hash</t>
@@ -831,6 +867,18 @@
   </si>
   <si>
     <t xml:space="preserve">lote_20260924_mob01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a66063dfa46994897ebd9b0ba858fdff59beaf63578cedd1cc72062f83e22f86</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-24T12:25:44</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2026-09-24, lote_20260924_ui01]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lote_20260924_ui01</t>
   </si>
 </sst>
 </file>
@@ -1326,11 +1374,11 @@
       </c>
       <c r="C4" s="3" t="n">
         <f aca="false">COUNTIF(Login!I2:I200,"Por testar")</f>
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="D4" s="3" t="n">
         <f aca="false">COUNTIF(Login!I2:I200,"Pass")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E4" s="3" t="n">
         <f aca="false">COUNTIF(Login!I2:I200,"Fail")</f>
@@ -1346,7 +1394,7 @@
       </c>
       <c r="H4" s="4" t="n">
         <f aca="false">IFERROR((B4-C4)/B4,0)</f>
-        <v>0</v>
+        <v>0.428571428571429</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1359,15 +1407,15 @@
       </c>
       <c r="C5" s="3" t="n">
         <f aca="false">COUNTIF(Produtos!I2:I200,"Por testar")</f>
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="D5" s="3" t="n">
         <f aca="false">COUNTIF(Produtos!I2:I200,"Pass")</f>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="E5" s="3" t="n">
         <f aca="false">COUNTIF(Produtos!I2:I200,"Fail")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F5" s="3" t="n">
         <f aca="false">COUNTIF(Produtos!I2:I200,"Blocked")</f>
@@ -1379,7 +1427,7 @@
       </c>
       <c r="H5" s="4" t="n">
         <f aca="false">IFERROR((B5-C5)/B5,0)</f>
-        <v>0</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1392,11 +1440,11 @@
       </c>
       <c r="C6" s="3" t="n">
         <f aca="false">COUNTIF(Checkout!I2:I200,"Por testar")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D6" s="3" t="n">
         <f aca="false">COUNTIF(Checkout!I2:I200,"Pass")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="3" t="n">
         <f aca="false">COUNTIF(Checkout!I2:I200,"Fail")</f>
@@ -1412,7 +1460,7 @@
       </c>
       <c r="H6" s="4" t="n">
         <f aca="false">IFERROR((B6-C6)/B6,0)</f>
-        <v>0</v>
+        <v>0.166666666666667</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1524,15 +1572,15 @@
       </c>
       <c r="C10" s="3" t="n">
         <f aca="false">SUM(C4:C9)</f>
-        <v>20</v>
+        <v>13</v>
       </c>
       <c r="D10" s="3" t="n">
         <f aca="false">SUM(D4:D9)</f>
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="E10" s="3" t="n">
         <f aca="false">SUM(E4:E9)</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F10" s="3" t="n">
         <f aca="false">SUM(F4:F9)</f>
@@ -1544,7 +1592,7 @@
       </c>
       <c r="H10" s="4" t="n">
         <f aca="false">IFERROR((B10-C10)/B10,0)</f>
-        <v>0.473684210526316</v>
+        <v>0.657894736842105</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1568,84 +1616,104 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>240</v>
+        <v>251</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>241</v>
+        <v>252</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>242</v>
+        <v>253</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>243</v>
+        <v>254</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>244</v>
+        <v>255</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>245</v>
+        <v>256</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>246</v>
+        <v>257</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>247</v>
+        <v>258</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>248</v>
+        <v>259</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>249</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>250</v>
+        <v>261</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>251</v>
+        <v>262</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>252</v>
+        <v>263</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>5</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>253</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>254</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>255</v>
-      </c>
-      <c r="C4" s="0" t="s">
-        <v>256</v>
-      </c>
-      <c r="D4" s="0" t="n">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>265</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>266</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>267</v>
+      </c>
+      <c r="D4" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="F4" s="0" t="s">
-        <v>257</v>
+      <c r="F4" s="3" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="s">
+        <v>269</v>
+      </c>
+      <c r="B5" s="0" t="s">
+        <v>270</v>
+      </c>
+      <c r="C5" s="0" t="s">
+        <v>271</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="E5" s="0" t="s">
+        <v>246</v>
+      </c>
+      <c r="F5" s="0" t="s">
+        <v>272</v>
       </c>
     </row>
   </sheetData>
@@ -1739,23 +1807,25 @@
         <v>34</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>35</v>
+      </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>31</v>
@@ -1767,51 +1837,55 @@
         <v>33</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J3" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>41</v>
+      </c>
       <c r="K3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>30</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F4" s="6" t="s">
         <v>32</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="I4" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J4" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="J4" s="6" t="s">
+        <v>48</v>
+      </c>
       <c r="K4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>29</v>
@@ -1820,16 +1894,16 @@
         <v>30</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F5" s="6" t="s">
         <v>32</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>3</v>
@@ -1839,10 +1913,10 @@
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>29</v>
@@ -1851,16 +1925,16 @@
         <v>30</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F6" s="6" t="s">
         <v>32</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>3</v>
@@ -1870,28 +1944,28 @@
     </row>
     <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>3</v>
@@ -1901,28 +1975,28 @@
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>3</v>
@@ -2579,10 +2653,10 @@
     </row>
     <row r="2" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>29</v>
@@ -2594,26 +2668,28 @@
         <v>31</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>73</v>
+      </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>29</v>
@@ -2622,29 +2698,31 @@
         <v>30</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="I3" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J3" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>78</v>
+      </c>
       <c r="K3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>29</v>
@@ -2653,16 +2731,16 @@
         <v>30</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>3</v>
@@ -2672,10 +2750,10 @@
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>29</v>
@@ -2684,16 +2762,16 @@
         <v>30</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>3</v>
@@ -2703,34 +2781,38 @@
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="I6" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J6" s="6"/>
-      <c r="K6" s="6"/>
+        <v>5</v>
+      </c>
+      <c r="J6" s="6" t="s">
+        <v>93</v>
+      </c>
+      <c r="K6" s="6" t="s">
+        <v>94</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="I7" s="7"/>
@@ -3387,59 +3469,61 @@
     </row>
     <row r="2" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="I2" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J2" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>99</v>
+      </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>93</v>
+        <v>101</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>95</v>
+        <v>103</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>3</v>
@@ -3449,10 +3533,10 @@
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>97</v>
+        <v>105</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>98</v>
+        <v>106</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>29</v>
@@ -3461,16 +3545,16 @@
         <v>30</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>99</v>
+        <v>107</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>3</v>
@@ -3480,10 +3564,10 @@
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>29</v>
@@ -3492,16 +3576,16 @@
         <v>30</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>3</v>
@@ -3511,28 +3595,28 @@
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>3</v>
@@ -3542,28 +3626,28 @@
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>94</v>
+        <v>102</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>3</v>
@@ -4223,13 +4307,13 @@
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>30</v>
@@ -4238,31 +4322,31 @@
         <v>31</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>30</v>
@@ -4271,31 +4355,31 @@
         <v>31</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="K3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D4" s="6" t="s">
         <v>30</v>
@@ -4304,252 +4388,252 @@
         <v>31</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="K4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="K5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>30</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="K6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>144</v>
+        <v>152</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>145</v>
+        <v>153</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>147</v>
+        <v>155</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>148</v>
+        <v>156</v>
       </c>
       <c r="K7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>149</v>
+        <v>157</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>150</v>
+        <v>158</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>154</v>
+        <v>162</v>
       </c>
       <c r="K8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>155</v>
+        <v>163</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>156</v>
+        <v>164</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>30</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>157</v>
+        <v>165</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>158</v>
+        <v>166</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>159</v>
+        <v>167</v>
       </c>
       <c r="K9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>161</v>
+        <v>169</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D10" s="6" t="s">
         <v>30</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>162</v>
+        <v>170</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>163</v>
+        <v>171</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>5</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>164</v>
+        <v>172</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>165</v>
+        <v>173</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>166</v>
+        <v>174</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>167</v>
+        <v>175</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E11" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>151</v>
+        <v>159</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>168</v>
+        <v>176</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>169</v>
+        <v>177</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>170</v>
+        <v>178</v>
       </c>
       <c r="K11" s="6"/>
     </row>
@@ -5193,160 +5277,160 @@
     </row>
     <row r="2" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>171</v>
+        <v>179</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>172</v>
+        <v>180</v>
       </c>
       <c r="C2" s="6" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>177</v>
+        <v>185</v>
       </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>178</v>
+        <v>186</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>179</v>
+        <v>187</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>181</v>
+        <v>189</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>182</v>
+        <v>190</v>
       </c>
       <c r="K3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>183</v>
+        <v>191</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>185</v>
+        <v>193</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>186</v>
+        <v>194</v>
       </c>
       <c r="K4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>187</v>
+        <v>195</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>188</v>
+        <v>196</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>180</v>
+        <v>188</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>176</v>
+        <v>184</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>190</v>
+        <v>198</v>
       </c>
       <c r="K5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>191</v>
+        <v>199</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>192</v>
+        <v>200</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>194</v>
+        <v>202</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>195</v>
+        <v>203</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>196</v>
+        <v>204</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>3</v>
@@ -5356,51 +5440,51 @@
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>198</v>
+        <v>206</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="E7" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>199</v>
+        <v>207</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>200</v>
+        <v>208</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>201</v>
+        <v>209</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>5</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>202</v>
+        <v>210</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>203</v>
+        <v>211</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>204</v>
+        <v>212</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>205</v>
+        <v>213</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>193</v>
+        <v>201</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>31</v>
@@ -5409,10 +5493,10 @@
         <v>32</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>206</v>
+        <v>214</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>207</v>
+        <v>215</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>3</v>
@@ -6069,10 +6153,10 @@
     </row>
     <row r="2" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>209</v>
+        <v>217</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>29</v>
@@ -6084,85 +6168,85 @@
         <v>31</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>211</v>
+        <v>219</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>212</v>
+        <v>220</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>213</v>
+        <v>221</v>
       </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>214</v>
+        <v>222</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>215</v>
+        <v>223</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>216</v>
+        <v>224</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>217</v>
+        <v>225</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>218</v>
+        <v>226</v>
       </c>
       <c r="K3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>219</v>
+        <v>227</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>220</v>
+        <v>228</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>210</v>
+        <v>218</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>221</v>
+        <v>229</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>223</v>
+        <v>231</v>
       </c>
       <c r="K4" s="6"/>
     </row>
@@ -6776,7 +6860,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6787,19 +6871,19 @@
         <v>17</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>224</v>
+        <v>232</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>20</v>
@@ -6808,80 +6892,115 @@
         <v>24</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>227</v>
+        <v>235</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>228</v>
+        <v>236</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>231</v>
+        <v>239</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>234</v>
+        <v>242</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>235</v>
+        <v>243</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>236</v>
+        <v>244</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>237</v>
+        <v>245</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>197</v>
+        <v>205</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>29</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>233</v>
+        <v>241</v>
       </c>
       <c r="K3" s="3" t="s">
-        <v>234</v>
+        <v>242</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="s">
+        <v>246</v>
+      </c>
+      <c r="B4" s="0" t="s">
+        <v>247</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>248</v>
+      </c>
+      <c r="D4" s="0" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="0" t="s">
+        <v>88</v>
+      </c>
+      <c r="F4" s="0" t="s">
+        <v>90</v>
+      </c>
+      <c r="G4" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="H4" s="0" t="s">
+        <v>45</v>
+      </c>
+      <c r="I4" s="0" t="s">
+        <v>240</v>
+      </c>
+      <c r="J4" s="0" t="s">
+        <v>241</v>
+      </c>
+      <c r="K4" s="0" t="s">
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -6900,17 +7019,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:H6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>238</v>
+        <v>249</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>239</v>
+        <v>250</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6921,7 +7040,7 @@
         <v>20</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>226</v>
+        <v>234</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>24</v>
@@ -6933,7 +7052,7 @@
         <v>17</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>225</v>
+        <v>233</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>18</v>
@@ -6941,53 +7060,79 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>229</v>
+        <v>237</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>12</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>230</v>
+        <v>238</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>160</v>
+        <v>168</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>235</v>
+        <v>246</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>76</v>
+        <v>45</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>232</v>
+        <v>240</v>
       </c>
       <c r="E5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="H5" s="3" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="E6" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="3" t="s">
-        <v>236</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>197</v>
-      </c>
-      <c r="H5" s="3" t="s">
+      <c r="F6" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="H6" s="3" t="s">
         <v>29</v>
       </c>
     </row>

</xml_diff>

<commit_message>
demo: decisoes do utilizador (delegacao aprovada, CT-LOGIN-006, 6.2)
- Aprovadas as decisoes tomadas por delegacao: casos de API, acessibilidade
  e mobile, BUG-1..3 com as prioridades propostas, .env com contas publicas.
- CT-LOGIN-006: Pass; esperado reescrito (o URL pode continuar
  /inventory.html); lote_20260924_ui02 e workbook reconstruido (26/38).
- 6.2: o repositorio fica privado por agora.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/demo/workbook/plano-demo.xlsx
+++ b/examples/demo/workbook/plano-demo.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="556" uniqueCount="273">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="278">
   <si>
     <t xml:space="preserve">Demo QA — saucedemo.com (site público de prática)</t>
   </si>
@@ -221,7 +221,10 @@
     <t xml:space="preserve">1. Abrir diretamente /inventory.html.</t>
   </si>
   <si>
-    <t xml:space="preserve">Volta à página de login com o erro "Epic sadface: You can only access '/inventory.html' when you are logged in.".</t>
+    <t xml:space="preserve">Mostra o formulário de login com o erro "Epic sadface: You can only access '/inventory.html' when you are logged in." (o URL pode continuar /inventory.html — decisão do utilizador, 24.09.2026).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sem sessão, /inventory.html mostra o formulário de login com "Epic sadface: You can only access '/inventory.html' when you are logged in."; o URL fica /inventory.html (aceite pelo esperado revisto). Observação da execução de 24.09.2026 (lote UI 01), reclassificada depois da resposta à Dúvida.</t>
   </si>
   <si>
     <t xml:space="preserve">CT-LOGIN-007</t>
@@ -836,7 +839,7 @@
     <t xml:space="preserve">5f9fd024e81cc1eab582ca9bdf73b0251242bd3c4c4d7ef356262b1d5494e6f8</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-24T12:15:59</t>
+    <t xml:space="preserve">2026-09-24T13:29:13</t>
   </si>
   <si>
     <t xml:space="preserve">[2026-09-24, lote_20260924_api01]</t>
@@ -848,7 +851,7 @@
     <t xml:space="preserve">1cb0929f96c97b3dbfd8cd74ffef5c07006ceeb02d0700501113aff216d6c4a6</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-24T12:16:01</t>
+    <t xml:space="preserve">2026-09-24T13:29:15</t>
   </si>
   <si>
     <t xml:space="preserve">[2026-09-24, lote_20260924_a11y01]</t>
@@ -860,7 +863,7 @@
     <t xml:space="preserve">80a1805992f0a3bb17024dd7f321d1a637283eb189d7343a34b6f27a61b246a8</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-24T12:16:04</t>
+    <t xml:space="preserve">2026-09-24T13:29:18</t>
   </si>
   <si>
     <t xml:space="preserve">[2026-09-24, lote_20260924_mob01]</t>
@@ -872,13 +875,25 @@
     <t xml:space="preserve">a66063dfa46994897ebd9b0ba858fdff59beaf63578cedd1cc72062f83e22f86</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-24T12:25:44</t>
+    <t xml:space="preserve">2026-09-24T13:29:20</t>
   </si>
   <si>
     <t xml:space="preserve">[2026-09-24, lote_20260924_ui01]</t>
   </si>
   <si>
     <t xml:space="preserve">lote_20260924_ui01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b25162c001d4fe6b4c098f024686d5ca6e599cacb703b6810a39ebecd53e6038</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-24T13:29:23</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2026-09-24, lote_20260924_ui02]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lote_20260924_ui02</t>
   </si>
 </sst>
 </file>
@@ -1374,11 +1389,11 @@
       </c>
       <c r="C4" s="3" t="n">
         <f aca="false">COUNTIF(Login!I2:I200,"Por testar")</f>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D4" s="3" t="n">
         <f aca="false">COUNTIF(Login!I2:I200,"Pass")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E4" s="3" t="n">
         <f aca="false">COUNTIF(Login!I2:I200,"Fail")</f>
@@ -1394,7 +1409,7 @@
       </c>
       <c r="H4" s="4" t="n">
         <f aca="false">IFERROR((B4-C4)/B4,0)</f>
-        <v>0.428571428571429</v>
+        <v>0.571428571428571</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1572,11 +1587,11 @@
       </c>
       <c r="C10" s="3" t="n">
         <f aca="false">SUM(C4:C9)</f>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D10" s="3" t="n">
         <f aca="false">SUM(D4:D9)</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E10" s="3" t="n">
         <f aca="false">SUM(E4:E9)</f>
@@ -1592,7 +1607,7 @@
       </c>
       <c r="H10" s="4" t="n">
         <f aca="false">IFERROR((B10-C10)/B10,0)</f>
-        <v>0.657894736842105</v>
+        <v>0.68421052631579</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1616,104 +1631,121 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F6"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="3" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>10</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>5</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>264</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>265</v>
+        <v>266</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>266</v>
+        <v>267</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>267</v>
+        <v>268</v>
       </c>
       <c r="D4" s="3" t="n">
         <v>3</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
         <v>269</v>
       </c>
-      <c r="B5" s="0" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>270</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="B5" s="3" t="s">
         <v>271</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="C5" s="3" t="s">
+        <v>272</v>
+      </c>
+      <c r="D5" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="E5" s="0" t="s">
-        <v>246</v>
-      </c>
-      <c r="F5" s="0" t="s">
-        <v>272</v>
+      <c r="E5" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="F5" s="3" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="s">
+        <v>274</v>
+      </c>
+      <c r="B6" s="0" t="s">
+        <v>275</v>
+      </c>
+      <c r="C6" s="0" t="s">
+        <v>276</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="0" t="s">
+        <v>277</v>
       </c>
     </row>
   </sheetData>
@@ -1942,7 +1974,7 @@
       <c r="J6" s="6"/>
       <c r="K6" s="6"/>
     </row>
-    <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
         <v>57</v>
       </c>
@@ -1968,35 +2000,37 @@
         <v>62</v>
       </c>
       <c r="I7" s="6" t="s">
-        <v>3</v>
-      </c>
-      <c r="J7" s="6"/>
+        <v>4</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>63</v>
+      </c>
       <c r="K7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>45</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>3</v>
@@ -2653,10 +2687,10 @@
     </row>
     <row r="2" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>29</v>
@@ -2668,28 +2702,28 @@
         <v>31</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>29</v>
@@ -2701,28 +2735,28 @@
         <v>45</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>29</v>
@@ -2731,16 +2765,16 @@
         <v>30</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>3</v>
@@ -2750,10 +2784,10 @@
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>29</v>
@@ -2765,13 +2799,13 @@
         <v>45</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>3</v>
@@ -2781,13 +2815,13 @@
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D6" s="6" t="s">
         <v>39</v>
@@ -2796,22 +2830,22 @@
         <v>45</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>5</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="K6" s="6" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3469,61 +3503,61 @@
     </row>
     <row r="2" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>45</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>3</v>
@@ -3533,10 +3567,10 @@
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>29</v>
@@ -3548,13 +3582,13 @@
         <v>45</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>3</v>
@@ -3564,10 +3598,10 @@
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>29</v>
@@ -3579,13 +3613,13 @@
         <v>45</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>3</v>
@@ -3595,28 +3629,28 @@
     </row>
     <row r="6" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>3</v>
@@ -3626,28 +3660,28 @@
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>3</v>
@@ -4307,10 +4341,10 @@
     </row>
     <row r="2" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>44</v>
@@ -4322,31 +4356,31 @@
         <v>31</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D3" s="6" t="s">
         <v>30</v>
@@ -4355,28 +4389,28 @@
         <v>31</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="K3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>44</v>
@@ -4388,61 +4422,61 @@
         <v>31</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="K4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>44</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="K5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>44</v>
@@ -4454,28 +4488,28 @@
         <v>45</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J6" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="K6" s="6"/>
     </row>
     <row r="7" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>44</v>
@@ -4487,64 +4521,64 @@
         <v>31</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="K7" s="6"/>
     </row>
     <row r="8" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F8" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J8" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="K8" s="6"/>
     </row>
     <row r="9" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D9" s="6" t="s">
         <v>30</v>
@@ -4553,28 +4587,28 @@
         <v>45</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="H9" s="6" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="I9" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J9" s="6" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="K9" s="6"/>
     </row>
     <row r="10" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C10" s="6" t="s">
         <v>44</v>
@@ -4586,54 +4620,54 @@
         <v>45</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="H10" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="I10" s="6" t="s">
         <v>5</v>
       </c>
       <c r="J10" s="6" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="K10" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="68.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="D11" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E11" s="6" t="s">
         <v>45</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="H11" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="I11" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J11" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="K11" s="6"/>
     </row>
@@ -5277,160 +5311,160 @@
     </row>
     <row r="2" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>44</v>
       </c>
       <c r="D2" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E2" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E3" s="6" t="s">
         <v>31</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="K3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>45</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="K4" s="6"/>
     </row>
     <row r="5" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C5" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>45</v>
       </c>
       <c r="F5" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="H5" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="I5" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J5" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="K5" s="6"/>
     </row>
     <row r="6" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C6" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D6" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>45</v>
       </c>
       <c r="F6" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="H6" s="6" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="I6" s="6" t="s">
         <v>3</v>
@@ -5440,51 +5474,51 @@
     </row>
     <row r="7" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="6" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="C7" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>45</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="H7" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="I7" s="6" t="s">
         <v>5</v>
       </c>
       <c r="J7" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="23.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="6" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="C8" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D8" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>31</v>
@@ -5493,10 +5527,10 @@
         <v>32</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="H8" s="6" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="I8" s="6" t="s">
         <v>3</v>
@@ -6153,10 +6187,10 @@
     </row>
     <row r="2" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="6" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>29</v>
@@ -6168,28 +6202,28 @@
         <v>31</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J2" s="6" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="K2" s="6"/>
     </row>
     <row r="3" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="6" t="s">
-        <v>222</v>
+        <v>223</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>223</v>
+        <v>224</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>38</v>
@@ -6201,52 +6235,52 @@
         <v>31</v>
       </c>
       <c r="F3" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="I3" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J3" s="6" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="K3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="6" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>29</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>45</v>
       </c>
       <c r="F4" s="6" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="I4" s="6" t="s">
         <v>4</v>
       </c>
       <c r="J4" s="6" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="K4" s="6"/>
     </row>
@@ -6871,19 +6905,19 @@
         <v>17</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="D1" s="2" t="s">
         <v>1</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>18</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="H1" s="2" t="s">
         <v>20</v>
@@ -6892,27 +6926,27 @@
         <v>24</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="C2" s="8" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>12</v>
       </c>
       <c r="E2" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F2" s="3" t="s">
         <v>44</v>
@@ -6924,83 +6958,83 @@
         <v>45</v>
       </c>
       <c r="I2" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="57" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="C3" s="8" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>13</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F3" s="3" t="s">
         <v>29</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="J3" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="K3" s="3" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="C4" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="I4" s="3" t="s">
         <v>241</v>
       </c>
-      <c r="K3" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>242</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
-        <v>246</v>
-      </c>
-      <c r="B4" s="0" t="s">
-        <v>247</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>248</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="E4" s="0" t="s">
-        <v>88</v>
-      </c>
-      <c r="F4" s="0" t="s">
-        <v>90</v>
-      </c>
-      <c r="G4" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="H4" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="I4" s="0" t="s">
-        <v>240</v>
-      </c>
-      <c r="J4" s="0" t="s">
-        <v>241</v>
-      </c>
-      <c r="K4" s="0" t="s">
-        <v>242</v>
+      <c r="K4" s="3" t="s">
+        <v>243</v>
       </c>
     </row>
   </sheetData>
@@ -7024,12 +7058,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="5" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7040,7 +7074,7 @@
         <v>20</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>24</v>
@@ -7052,7 +7086,7 @@
         <v>17</v>
       </c>
       <c r="G3" s="2" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="H3" s="2" t="s">
         <v>18</v>
@@ -7060,7 +7094,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>45</v>
@@ -7069,16 +7103,16 @@
         <v>45</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E4" s="3" t="s">
         <v>12</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="H4" s="3" t="s">
         <v>44</v>
@@ -7086,7 +7120,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>45</v>
@@ -7095,42 +7129,42 @@
         <v>45</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E5" s="3" t="s">
         <v>10</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="E6" s="3" t="s">
         <v>13</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="H6" s="3" t="s">
         <v>29</v>

</xml_diff>

<commit_message>
7.6: demo reproduzivel (aplicar --agora e teste da reconstrucao no CI)
- ExcelAdapter.agora / aplicar --agora: datas escritas fixas (etiqueta, data
  de report, resumo da vista, aplicado_em); sem a opcao, o relogio
- reconstruir_workbook.py usa o 1.o ts de cada lote e aceita outra pasta
- tests/test_demo_reproduzivel.py; a parte com LibreOffice corre no job golden
- workbook do demo regenerado com as datas de execucao dos lotes

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/demo/workbook/plano-demo.xlsx
+++ b/examples/demo/workbook/plano-demo.xlsx
@@ -839,55 +839,55 @@
     <t xml:space="preserve">5f9fd024e81cc1eab582ca9bdf73b0251242bd3c4c4d7ef356262b1d5494e6f8</t>
   </si>
   <si>
+    <t xml:space="preserve">2026-09-24T11:31:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2026-09-24, lote_20260924_api01]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lote_20260924_api01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1cb0929f96c97b3dbfd8cd74ffef5c07006ceeb02d0700501113aff216d6c4a6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-24T11:31:03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2026-09-24, lote_20260924_a11y01]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lote_20260924_a11y01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">80a1805992f0a3bb17024dd7f321d1a637283eb189d7343a34b6f27a61b246a8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-24T12:13:46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2026-09-24, lote_20260924_mob01]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lote_20260924_mob01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">a66063dfa46994897ebd9b0ba858fdff59beaf63578cedd1cc72062f83e22f86</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-09-24T12:24:30</t>
+  </si>
+  <si>
+    <t xml:space="preserve">[2026-09-24, lote_20260924_ui01]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lote_20260924_ui01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">b25162c001d4fe6b4c098f024686d5ca6e599cacb703b6810a39ebecd53e6038</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-09-24T13:29:13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[2026-09-24, lote_20260924_api01]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lote_20260924_api01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1cb0929f96c97b3dbfd8cd74ffef5c07006ceeb02d0700501113aff216d6c4a6</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-24T13:29:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[2026-09-24, lote_20260924_a11y01]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lote_20260924_a11y01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">80a1805992f0a3bb17024dd7f321d1a637283eb189d7343a34b6f27a61b246a8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-24T13:29:18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[2026-09-24, lote_20260924_mob01]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lote_20260924_mob01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">a66063dfa46994897ebd9b0ba858fdff59beaf63578cedd1cc72062f83e22f86</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-24T13:29:20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">[2026-09-24, lote_20260924_ui01]</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lote_20260924_ui01</t>
-  </si>
-  <si>
-    <t xml:space="preserve">b25162c001d4fe6b4c098f024686d5ca6e599cacb703b6810a39ebecd53e6038</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-09-24T13:29:23</t>
   </si>
   <si>
     <t xml:space="preserve">[2026-09-24, lote_20260924_ui02]</t>

</xml_diff>